<commit_message>
Save library recording Session 28 Oct 2026 4:48:42 PM - 5d8b674f-2cf5-46e6-aba4-db9e6801e885 - 2026-10-28T05:53:57.708544Z
</commit_message>
<xml_diff>
--- a/library/projects/6e6f2be2-b3ee-4194-9cb9-2a3d21e6008e/recordings/5d8b674f-2cf5-46e6-aba4-db9e6801e885/resources/azure-devops.xlsx
+++ b/library/projects/6e6f2be2-b3ee-4194-9cb9-2a3d21e6008e/recordings/5d8b674f-2cf5-46e6-aba4-db9e6801e885/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,494 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://www.harrisfarm.com.au/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.harrisfarm.com.au/</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Click DELIVERY</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-find-flow &gt; div:nth-of-type(1) &gt; button:nth-of-type(3)", "x": 416, "y": 509, "text": "DELIVERY", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>step-002.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Click e.g. 2066</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{"primary": "input[name=\"postcode\"]", "x": 460, "y": 472, "text": "e.g. 2066", "tag": "input"}</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>step-003.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Type: 2047</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2047</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{"primary": "input[name=\"postcode\"]"}</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>step-004.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Click CHECK DELIVERY</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-find", "x": 675, "y": 464, "text": "CHECK DELIVERY", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>step-005.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Click CONTINUE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"primary": "#store-picker-select-slot", "x": 385, "y": 535, "text": "CONTINUE", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>step-006.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Click 29 Oct</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-days &gt; button:nth-of-type(2) &gt; span:nth-of-type(2)", "x": 460, "y": 205, "text": "29 Oct", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>step-007.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Click Afternoon</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-periods &gt; button:nth-of-type(2)", "x": 484, "y": 255, "text": "Afternoon", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>step-008.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Click 12:00 PM-1:00 PM
+12:30 PM-1:30 PM
+1:00 PM-2:00 PM
+1:30 PM-2:30 PM
+2:00 PM-3:00 P</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-slots", "x": 437, "y": 409, "text": "12:00 PM-1:00 PM\n12:30 PM-1:30 PM\n1:00 PM-2:00 PM\n1:30 PM-2:30 PM\n2:00 PM-3:00 P", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>step-009.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Click 12:30 PM-1:30 PM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-slots &gt; button:nth-of-type(2) &gt; span:nth-of-type(1)", "x": 453, "y": 381, "text": "12:30 PM-1:30 PM", "tag": "span"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>step-010.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Click RESERVE TIME</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"primary": "#cart-slot-reserve", "x": 623, "y": 579, "text": "RESERVE TIME", "tag": "button"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Click Shop promotion item 3</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{"primary": "a[aria-label=\"Shop promotion item 3\"]", "x": 678, "y": 425, "text": "Shop promotion item 3", "tag": "a"}</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Click 654,349</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{"primary": "section:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(2) &gt; product-info:nth-of-type(1) &gt; div:nth-of-type(2) &gt; div:nth-of-type(2)", "x": 654, "y": 349, "text": "", "tag": "div"}</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>step-013.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Click 649,394</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{"primary": null, "x": 649, "y": 394, "text": null, "tag": null}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>step-014.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Click 107,80</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{"primary": "header:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; a:nth-of-type(1) &gt; img:nth-of-type(1)", "x": 107, "y": 80, "text": "", "tag": "img"}</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Click 97,48</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{"primary": "div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; div:nth-of-type(1) &gt; h1:nth-of-type(1) &gt; a:nth-of-type(1) &gt; img:nth-of-type(1)", "x": 97, "y": 48, "text": "", "tag": "img"}</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Click 934,74</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{"primary": null, "x": 934, "y": 74, "text": null, "tag": null}</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Session 28 Oct 2026 4:48:42 PM</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Click Shop promotion item 3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{"primary": "a[aria-label=\"Shop promotion item 3\"]", "x": 698, "y": 404, "text": "Shop promotion item 3", "tag": "a"}</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>